<commit_message>
Update Problem 4 21/10
</commit_message>
<xml_diff>
--- a/Problem 4/TF_Parameters.xlsx
+++ b/Problem 4/TF_Parameters.xlsx
@@ -15,13 +15,15 @@
   <sheets>
     <sheet name="Deterministic 1st Order" sheetId="1" r:id="rId1"/>
     <sheet name="Stochastic 1st Order" sheetId="3" r:id="rId2"/>
+    <sheet name="Deterministic 2nd Order" sheetId="4" r:id="rId6"/>
+    <sheet name="Stochastic 2nd Order" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="396" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="522" uniqueCount="13">
   <si>
     <t>TransferFunction</t>
   </si>
@@ -54,6 +56,12 @@
   </si>
   <si>
     <t>G42</t>
+  </si>
+  <si>
+    <t>Tau1_s</t>
+  </si>
+  <si>
+    <t>Tau2_s</t>
   </si>
 </sst>
 </file>
@@ -562,10 +570,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>0.21577613660737197</v>
+        <v>0.20245939154354964</v>
       </c>
       <c r="C2" s="0">
-        <v>174.76359658211501</v>
+        <v>146.35286081533505</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
@@ -573,10 +581,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>0.12881968843818181</v>
+        <v>0.10896474055679183</v>
       </c>
       <c r="C3" s="0">
-        <v>279.51478537738473</v>
+        <v>237.77055610486616</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
@@ -584,10 +592,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>0.16011818092593047</v>
+        <v>0.15140391722786242</v>
       </c>
       <c r="C4" s="0">
-        <v>306.35003683037371</v>
+        <v>253.33825876419755</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
@@ -595,10 +603,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>0.25208607993299942</v>
+        <v>0.25509143119565181</v>
       </c>
       <c r="C5" s="0">
-        <v>133.74355924842379</v>
+        <v>140.91158095296001</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
@@ -606,10 +614,10 @@
         <v>7</v>
       </c>
       <c r="B6" s="0">
-        <v>0.0099074292031426682</v>
+        <v>0.0039616682534490437</v>
       </c>
       <c r="C6" s="0">
-        <v>123.22645885432243</v>
+        <v>123.05302438540853</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
@@ -617,10 +625,10 @@
         <v>8</v>
       </c>
       <c r="B7" s="0">
-        <v>0.065121861771454084</v>
+        <v>0.060528088905640071</v>
       </c>
       <c r="C7" s="0">
-        <v>90.697912922583697</v>
+        <v>83.484996678797799</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
@@ -628,10 +636,10 @@
         <v>9</v>
       </c>
       <c r="B8" s="0">
-        <v>0.082868009361191861</v>
+        <v>0.084984765735841433</v>
       </c>
       <c r="C8" s="0">
-        <v>46.546443659500454</v>
+        <v>78.753942061356398</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
@@ -639,13 +647,295 @@
         <v>10</v>
       </c>
       <c r="B9" s="0">
-        <v>0.0034948517564782696</v>
+        <v>0.001397864390268979</v>
       </c>
       <c r="C9" s="0">
-        <v>3.1235830797932698</v>
+        <v>3.151803677376297</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.77734375" customWidth="true"/>
+    <col min="2" max="2" width="15.88671875" customWidth="true"/>
+    <col min="3" max="3" width="11.5546875" customWidth="true"/>
+    <col min="4" max="4" width="11.5546875" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>0.18427533609698565</v>
+      </c>
+      <c r="C2" s="0">
+        <v>11.982700083595699</v>
+      </c>
+      <c r="D2" s="0">
+        <v>116.57787272981868</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>0.091082044272262242</v>
+      </c>
+      <c r="C3" s="0">
+        <v>100.63548518267035</v>
+      </c>
+      <c r="D3" s="0">
+        <v>100.63548518267035</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>0.13808778975393415</v>
+      </c>
+      <c r="C4" s="0">
+        <v>109.53433377660443</v>
+      </c>
+      <c r="D4" s="0">
+        <v>109.53433377660443</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>0.24410260374243761</v>
+      </c>
+      <c r="C5" s="0">
+        <v>11.765260352474582</v>
+      </c>
+      <c r="D5" s="0">
+        <v>132.72780015592389</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="0">
+        <v>-4.8831374818328504e-09</v>
+      </c>
+      <c r="C6" s="0">
+        <v>60.267348585448694</v>
+      </c>
+      <c r="D6" s="0">
+        <v>66.144238613417713</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="0">
+        <v>0.054670662042947939</v>
+      </c>
+      <c r="C7" s="0">
+        <v>13.481254983358317</v>
+      </c>
+      <c r="D7" s="0">
+        <v>66.742279564031534</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="0">
+        <v>0.081431577500194904</v>
+      </c>
+      <c r="C8" s="0">
+        <v>12.981820631868416</v>
+      </c>
+      <c r="D8" s="0">
+        <v>75.797431906884214</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="0">
+        <v>4.1207607319593377e-08</v>
+      </c>
+      <c r="C9" s="0">
+        <v>8.105818908866917</v>
+      </c>
+      <c r="D9" s="0">
+        <v>634.03124311599356</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.77734375" customWidth="true"/>
+    <col min="2" max="2" width="14.5546875" customWidth="true"/>
+    <col min="3" max="3" width="15.5546875" customWidth="true"/>
+    <col min="4" max="4" width="15.5546875" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>0.2026241352411951</v>
+      </c>
+      <c r="C2" s="0">
+        <v>0.019869986689005657</v>
+      </c>
+      <c r="D2" s="0">
+        <v>151.3141175348099</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>0.10559334280905984</v>
+      </c>
+      <c r="C3" s="0">
+        <v>73.259712926623365</v>
+      </c>
+      <c r="D3" s="0">
+        <v>156.88922503834672</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>0.15116367517131199</v>
+      </c>
+      <c r="C4" s="0">
+        <v>1.7842731021636311</v>
+      </c>
+      <c r="D4" s="0">
+        <v>249.95201816536925</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>0.25763123795620441</v>
+      </c>
+      <c r="C5" s="0">
+        <v>0.4819792235854311</v>
+      </c>
+      <c r="D5" s="0">
+        <v>156.89255155776661</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="0">
+        <v>0.0021806702705690875</v>
+      </c>
+      <c r="C6" s="0">
+        <v>6855263227117297</v>
+      </c>
+      <c r="D6" s="0">
+        <v>6855263227117297</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="0">
+        <v>0.059299615203499599</v>
+      </c>
+      <c r="C7" s="0">
+        <v>96.019044676232838</v>
+      </c>
+      <c r="D7" s="0">
+        <v>96.019044676232838</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="0">
+        <v>0.087080723932905738</v>
+      </c>
+      <c r="C8" s="0">
+        <v>108.09075402654523</v>
+      </c>
+      <c r="D8" s="0">
+        <v>261.81902378484813</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="0">
+        <v>0.0011076473168078389</v>
+      </c>
+      <c r="C9" s="0">
+        <v>1350.2034201405593</v>
+      </c>
+      <c r="D9" s="0">
+        <v>1350.2034201405593</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update Problem 4 23/10
</commit_message>
<xml_diff>
--- a/Problem 4/TF_Parameters.xlsx
+++ b/Problem 4/TF_Parameters.xlsx
@@ -8,22 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Documents\MIGUEL\Miguel Faculdade\5º Ano\DTU\MPC\02619---MPC-project\Problem 4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2E486B6-E5F4-45CF-B6F6-AD44BC096BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{242FA3C5-4B3E-4A7A-9DBE-B14F71B98925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="8880"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Deterministic 1st Order" sheetId="1" r:id="rId1"/>
     <sheet name="Stochastic 1st Order" sheetId="3" r:id="rId2"/>
-    <sheet name="Deterministic 2nd Order" sheetId="4" r:id="rId6"/>
-    <sheet name="Stochastic 2nd Order" sheetId="5" r:id="rId7"/>
+    <sheet name="Deterministic 2nd Order" sheetId="4" r:id="rId3"/>
+    <sheet name="Stochastic 2nd Order" sheetId="5" r:id="rId4"/>
+    <sheet name="Deterministic Delay" sheetId="8" r:id="rId5"/>
+    <sheet name="Stochastic Delay" sheetId="9" r:id="rId6"/>
+    <sheet name="Deterministic RMSE" sheetId="6" r:id="rId7"/>
+    <sheet name="Stochastic RMSE" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="522" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="470" uniqueCount="17">
   <si>
     <t>TransferFunction</t>
   </si>
@@ -62,6 +66,18 @@
   </si>
   <si>
     <t>Tau2_s</t>
+  </si>
+  <si>
+    <t>RMSE_1st</t>
+  </si>
+  <si>
+    <t>RMSE_2nd</t>
+  </si>
+  <si>
+    <t>Delay_s</t>
+  </si>
+  <si>
+    <t>RMSE_1st_Delay</t>
   </si>
 </sst>
 </file>
@@ -659,9 +675,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="true"/>
     <col min="2" max="2" width="15.88671875" customWidth="true"/>
@@ -669,7 +685,7 @@
     <col min="4" max="4" width="11.5546875" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
       <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
@@ -683,7 +699,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2" s="0" t="s">
         <v>1</v>
       </c>
@@ -697,7 +713,7 @@
         <v>116.57787272981868</v>
       </c>
     </row>
-    <row r="3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3" s="0" t="s">
         <v>2</v>
       </c>
@@ -711,7 +727,7 @@
         <v>100.63548518267035</v>
       </c>
     </row>
-    <row r="4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4" s="0" t="s">
         <v>3</v>
       </c>
@@ -725,7 +741,7 @@
         <v>109.53433377660443</v>
       </c>
     </row>
-    <row r="5">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
       <c r="A5" s="0" t="s">
         <v>4</v>
       </c>
@@ -739,7 +755,7 @@
         <v>132.72780015592389</v>
       </c>
     </row>
-    <row r="6">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
       <c r="A6" s="0" t="s">
         <v>7</v>
       </c>
@@ -753,7 +769,7 @@
         <v>66.144238613417713</v>
       </c>
     </row>
-    <row r="7">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
       <c r="A7" s="0" t="s">
         <v>8</v>
       </c>
@@ -767,7 +783,7 @@
         <v>66.742279564031534</v>
       </c>
     </row>
-    <row r="8">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
       <c r="A8" s="0" t="s">
         <v>9</v>
       </c>
@@ -781,7 +797,7 @@
         <v>75.797431906884214</v>
       </c>
     </row>
-    <row r="9">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
       <c r="A9" s="0" t="s">
         <v>10</v>
       </c>
@@ -796,13 +812,14 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="true"/>
     <col min="2" max="2" width="14.5546875" customWidth="true"/>
@@ -810,7 +827,7 @@
     <col min="4" max="4" width="15.5546875" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
       <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
@@ -824,7 +841,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2" s="0" t="s">
         <v>1</v>
       </c>
@@ -838,7 +855,7 @@
         <v>151.3141175348099</v>
       </c>
     </row>
-    <row r="3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3" s="0" t="s">
         <v>2</v>
       </c>
@@ -852,7 +869,7 @@
         <v>156.88922503834672</v>
       </c>
     </row>
-    <row r="4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4" s="0" t="s">
         <v>3</v>
       </c>
@@ -866,7 +883,7 @@
         <v>249.95201816536925</v>
       </c>
     </row>
-    <row r="5">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
       <c r="A5" s="0" t="s">
         <v>4</v>
       </c>
@@ -880,7 +897,7 @@
         <v>156.89255155776661</v>
       </c>
     </row>
-    <row r="6">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
       <c r="A6" s="0" t="s">
         <v>7</v>
       </c>
@@ -894,7 +911,7 @@
         <v>6855263227117297</v>
       </c>
     </row>
-    <row r="7">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
       <c r="A7" s="0" t="s">
         <v>8</v>
       </c>
@@ -908,7 +925,7 @@
         <v>96.019044676232838</v>
       </c>
     </row>
-    <row r="8">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
       <c r="A8" s="0" t="s">
         <v>9</v>
       </c>
@@ -922,7 +939,7 @@
         <v>261.81902378484813</v>
       </c>
     </row>
-    <row r="9">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
       <c r="A9" s="0" t="s">
         <v>10</v>
       </c>
@@ -937,5 +954,574 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.77734375" customWidth="true"/>
+    <col min="2" max="2" width="15.21875" customWidth="true"/>
+    <col min="3" max="3" width="11.5546875" customWidth="true"/>
+    <col min="4" max="4" width="7.33203125" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>0.18455203468866102</v>
+      </c>
+      <c r="C2" s="0">
+        <v>121.37637040490891</v>
+      </c>
+      <c r="D2" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
+      <c r="A3" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>0.092537915817242258</v>
+      </c>
+      <c r="C3" s="0">
+        <v>168.1898901641614</v>
+      </c>
+      <c r="D3" s="0">
+        <v>40</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
+      <c r="A4" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>0.14095878212341872</v>
+      </c>
+      <c r="C4" s="0">
+        <v>195.38018869166123</v>
+      </c>
+      <c r="D4" s="0">
+        <v>40</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
+      <c r="A5" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>0.24447031251160076</v>
+      </c>
+      <c r="C5" s="0">
+        <v>137.24276942490897</v>
+      </c>
+      <c r="D5" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
+      <c r="A6" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="0">
+        <v>4.8274890842975713e-09</v>
+      </c>
+      <c r="C6" s="0">
+        <v>23.692593188913669</v>
+      </c>
+      <c r="D6" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
+      <c r="A7" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="0">
+        <v>0.054764579680816591</v>
+      </c>
+      <c r="C7" s="0">
+        <v>73.553721187212489</v>
+      </c>
+      <c r="D7" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
+      <c r="A8" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="0">
+        <v>0.081563491011448594</v>
+      </c>
+      <c r="C8" s="0">
+        <v>81.952096128254453</v>
+      </c>
+      <c r="D8" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
+      <c r="A9" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="0">
+        <v>3.3865839478922294e-08</v>
+      </c>
+      <c r="C9" s="0">
+        <v>30.770723649179079</v>
+      </c>
+      <c r="D9" s="0">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.77734375" customWidth="true"/>
+    <col min="2" max="2" width="14.5546875" customWidth="true"/>
+    <col min="3" max="3" width="11.5546875" customWidth="true"/>
+    <col min="4" max="4" width="7.33203125" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>0.19898459747837935</v>
+      </c>
+      <c r="C2" s="0">
+        <v>80.564307219708752</v>
+      </c>
+      <c r="D2" s="0">
+        <v>80</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
+      <c r="A3" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>0.10432471870882548</v>
+      </c>
+      <c r="C3" s="0">
+        <v>134.9859008245603</v>
+      </c>
+      <c r="D3" s="0">
+        <v>104</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
+      <c r="A4" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>0.14659545488773584</v>
+      </c>
+      <c r="C4" s="0">
+        <v>154.5151108437999</v>
+      </c>
+      <c r="D4" s="0">
+        <v>116</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
+      <c r="A5" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>0.25509143119565181</v>
+      </c>
+      <c r="C5" s="0">
+        <v>140.91158095296001</v>
+      </c>
+      <c r="D5" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
+      <c r="A6" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="0">
+        <v>0.0039881053022574739</v>
+      </c>
+      <c r="C6" s="0">
+        <v>67.309092716161047</v>
+      </c>
+      <c r="D6" s="0">
+        <v>116</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
+      <c r="A7" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="0">
+        <v>0.059899840241413073</v>
+      </c>
+      <c r="C7" s="0">
+        <v>27.245552640263366</v>
+      </c>
+      <c r="D7" s="0">
+        <v>76</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
+      <c r="A8" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="0">
+        <v>0.083363794325083715</v>
+      </c>
+      <c r="C8" s="0">
+        <v>28.557231329151652</v>
+      </c>
+      <c r="D8" s="0">
+        <v>36</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
+      <c r="A9" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="0">
+        <v>0.0012947600074376228</v>
+      </c>
+      <c r="C9" s="0">
+        <v>775.5301922890734</v>
+      </c>
+      <c r="D9" s="0">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.77734375" customWidth="true"/>
+    <col min="2" max="2" width="15.21875" customWidth="true"/>
+    <col min="3" max="3" width="15.5546875" customWidth="true"/>
+    <col min="4" max="4" width="15.5546875" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>0.0028964223664025798</v>
+      </c>
+      <c r="C2" s="0">
+        <v>0.00058838173992153096</v>
+      </c>
+      <c r="D2" s="0">
+        <v>0.0012032585050254</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
+      <c r="A3" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>0.0049201328709937648</v>
+      </c>
+      <c r="C3" s="0">
+        <v>0.00096753978387204259</v>
+      </c>
+      <c r="D3" s="0">
+        <v>0.0018932720483514289</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
+      <c r="A4" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>0.0074987651601533248</v>
+      </c>
+      <c r="C4" s="0">
+        <v>0.001370448893248797</v>
+      </c>
+      <c r="D4" s="0">
+        <v>0.0030805226900424911</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
+      <c r="A5" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>0.0036496552388562919</v>
+      </c>
+      <c r="C5" s="0">
+        <v>0.00073680431052307544</v>
+      </c>
+      <c r="D5" s="0">
+        <v>0.0014868869911686964</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
+      <c r="A6" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="0">
+        <v>2.8111333571748617e-10</v>
+      </c>
+      <c r="C6" s="0">
+        <v>9.2103903490721472e-09</v>
+      </c>
+      <c r="D6" s="0">
+        <v>2.8111333571748617e-10</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
+      <c r="A7" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="0">
+        <v>0.0010746831755359442</v>
+      </c>
+      <c r="C7" s="0">
+        <v>0.00027401736504944064</v>
+      </c>
+      <c r="D7" s="0">
+        <v>0.00051567727392938566</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
+      <c r="A8" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="0">
+        <v>0.0015116884407328404</v>
+      </c>
+      <c r="C8" s="0">
+        <v>0.00035067457764949344</v>
+      </c>
+      <c r="D8" s="0">
+        <v>0.00069200418415255754</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
+      <c r="A9" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="0">
+        <v>1.9101688765403024e-09</v>
+      </c>
+      <c r="C9" s="0">
+        <v>1.3703136776879962e-08</v>
+      </c>
+      <c r="D9" s="0">
+        <v>1.9101688765403024e-09</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.77734375" customWidth="true"/>
+    <col min="2" max="2" width="13.5546875" customWidth="true"/>
+    <col min="4" max="4" width="14.6640625" customWidth="true"/>
+    <col min="3" max="3" width="13.5546875" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>0.01448964232638713</v>
+      </c>
+      <c r="C2" s="0">
+        <v>0.014500302956545853</v>
+      </c>
+      <c r="D2" s="0">
+        <v>0.023613150414056237</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
+      <c r="A3" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>0.015428771443546133</v>
+      </c>
+      <c r="C3" s="0">
+        <v>0.014437848951245077</v>
+      </c>
+      <c r="D3" s="0">
+        <v>0.015141207796765465</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
+      <c r="A4" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>0.013793434951433665</v>
+      </c>
+      <c r="C4" s="0">
+        <v>0.013784873522713126</v>
+      </c>
+      <c r="D4" s="0">
+        <v>0.020373396345811805</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
+      <c r="A5" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>0.015087443820643327</v>
+      </c>
+      <c r="C5" s="0">
+        <v>0.015905228292835718</v>
+      </c>
+      <c r="D5" s="0">
+        <v>0.015087443820643327</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
+      <c r="A6" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="0">
+        <v>0.015296640747141427</v>
+      </c>
+      <c r="C6" s="0">
+        <v>0.015073652361995997</v>
+      </c>
+      <c r="D6" s="0">
+        <v>0.01523068830150065</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
+      <c r="A7" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="0">
+        <v>0.015343651598767796</v>
+      </c>
+      <c r="C7" s="0">
+        <v>0.015124841236409449</v>
+      </c>
+      <c r="D7" s="0">
+        <v>0.01600236781736742</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
+      <c r="A8" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="0">
+        <v>0.014357583289211325</v>
+      </c>
+      <c r="C8" s="0">
+        <v>0.029728716893282648</v>
+      </c>
+      <c r="D8" s="0">
+        <v>0.015440563228031794</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
+      <c r="A9" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="0">
+        <v>0.014218302040384271</v>
+      </c>
+      <c r="C9" s="0">
+        <v>0.01440356581133953</v>
+      </c>
+      <c r="D9" s="0">
+        <v>0.014239799843973253</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>